<commit_message>
nmv 10 04 2026
</commit_message>
<xml_diff>
--- a/TS Jatai Working/Padam Input Templates/TS 6.6 Padam Input Template.xlsx
+++ b/TS Jatai Working/Padam Input Templates/TS 6.6 Padam Input Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ALL IMP DATA\GitHub\texts\TS Jatai Working\Padam Input Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB1D6E2-E6B3-4B05-B0E8-AAB3337FC576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{688517B3-D1AA-445B-9179-55AFE3C95871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3273,9 +3273,6 @@
     <t>aqgniqvatItya#gni - vati#</t>
   </si>
   <si>
-    <t>apa#bar.hiShaq ityapa# - baqraq.hiqShaqH</t>
-  </si>
-  <si>
     <t>praqyAqjAniti# pra - yAqjAn</t>
   </si>
   <si>
@@ -4009,6 +4006,9 @@
   </si>
   <si>
     <t>uqpAq(gm)qSu</t>
+  </si>
+  <si>
+    <t>apa#bar.hiShaq ityapa# - baqrq.hiqShaqH</t>
   </si>
 </sst>
 </file>
@@ -6812,7 +6812,7 @@
         <v>38</v>
       </c>
       <c r="N39" s="43" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="O39" s="8" t="s">
         <v>64</v>
@@ -7183,7 +7183,7 @@
         <v>85</v>
       </c>
       <c r="T48" s="15" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="U48" s="15"/>
       <c r="V48" s="42"/>
@@ -8136,7 +8136,7 @@
     </row>
     <row r="73" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="C73" s="10"/>
       <c r="D73" s="21"/>
@@ -9137,7 +9137,7 @@
       <c r="S100" s="8"/>
       <c r="T100" s="8"/>
       <c r="U100" s="8" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="V100" s="42"/>
     </row>
@@ -9917,7 +9917,7 @@
     </row>
     <row r="121" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="D121" s="22"/>
       <c r="H121" s="49" t="s">
@@ -11504,7 +11504,7 @@
         <v>85</v>
       </c>
       <c r="T167" s="8" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="U167" s="8"/>
       <c r="V167" s="42"/>
@@ -13975,7 +13975,7 @@
         <v>238</v>
       </c>
       <c r="N239" s="42" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="O239" s="7"/>
       <c r="P239" s="8" t="s">
@@ -13987,7 +13987,7 @@
       <c r="T239" s="8"/>
       <c r="U239" s="8"/>
       <c r="V239" s="42" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="240" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -17522,7 +17522,7 @@
     </row>
     <row r="343" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A343" s="60" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="D343" s="22"/>
       <c r="F343" s="50" t="s">
@@ -17550,7 +17550,7 @@
         <v>104</v>
       </c>
       <c r="N343" s="60" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="O343" s="8" t="s">
         <v>64</v>
@@ -18801,10 +18801,10 @@
       <c r="Q378" s="8"/>
       <c r="R378" s="8"/>
       <c r="S378" s="8" t="s">
+        <v>1293</v>
+      </c>
+      <c r="T378" s="8" t="s">
         <v>1294</v>
-      </c>
-      <c r="T378" s="8" t="s">
-        <v>1295</v>
       </c>
       <c r="U378" s="8"/>
       <c r="V378" s="42"/>
@@ -19947,7 +19947,7 @@
         <v>31</v>
       </c>
       <c r="N411" s="43" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="O411" s="7"/>
       <c r="P411" s="8"/>
@@ -22299,8 +22299,8 @@
       <c r="S479" s="8"/>
       <c r="T479" s="8"/>
       <c r="U479" s="8"/>
-      <c r="V479" s="42" t="s">
-        <v>1081</v>
+      <c r="V479" s="43" t="s">
+        <v>1322</v>
       </c>
     </row>
     <row r="480" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -22337,7 +22337,7 @@
       <c r="T480" s="8"/>
       <c r="U480" s="8"/>
       <c r="V480" s="42" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="481" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -22406,7 +22406,7 @@
       <c r="T482" s="8"/>
       <c r="U482" s="8"/>
       <c r="V482" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="483" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -22509,7 +22509,7 @@
       <c r="T485" s="8"/>
       <c r="U485" s="8"/>
       <c r="V485" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="486" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -22579,7 +22579,7 @@
       <c r="T487" s="8"/>
       <c r="U487" s="8"/>
       <c r="V487" s="42" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="488" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -22649,7 +22649,7 @@
       <c r="T489" s="8"/>
       <c r="U489" s="8"/>
       <c r="V489" s="42" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="490" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -22785,7 +22785,7 @@
       <c r="T493" s="8"/>
       <c r="U493" s="8"/>
       <c r="V493" s="43" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="494" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -22853,7 +22853,7 @@
         <v>85</v>
       </c>
       <c r="T495" s="8" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="U495" s="8"/>
       <c r="V495" s="42"/>
@@ -22991,7 +22991,7 @@
       <c r="T499" s="8"/>
       <c r="U499" s="8"/>
       <c r="V499" s="42" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="500" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -23127,7 +23127,7 @@
       <c r="T503" s="8"/>
       <c r="U503" s="8"/>
       <c r="V503" s="42" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="504" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -23300,7 +23300,7 @@
       <c r="T508" s="8"/>
       <c r="U508" s="8"/>
       <c r="V508" s="42" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="509" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -23370,7 +23370,7 @@
       <c r="T510" s="8"/>
       <c r="U510" s="8"/>
       <c r="V510" s="43" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="511" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -23407,7 +23407,7 @@
       <c r="T511" s="8"/>
       <c r="U511" s="8"/>
       <c r="V511" s="42" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="512" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -23477,7 +23477,7 @@
       <c r="T513" s="8"/>
       <c r="U513" s="8"/>
       <c r="V513" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="514" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -23580,7 +23580,7 @@
       <c r="T516" s="8"/>
       <c r="U516" s="8"/>
       <c r="V516" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="517" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -23650,7 +23650,7 @@
       <c r="T518" s="8"/>
       <c r="U518" s="8"/>
       <c r="V518" s="42" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="519" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -23763,7 +23763,7 @@
       </c>
       <c r="U521" s="8"/>
       <c r="V521" s="42" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="522" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -23870,7 +23870,7 @@
       <c r="T524" s="8"/>
       <c r="U524" s="8"/>
       <c r="V524" s="42" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="525" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -24240,7 +24240,7 @@
       <c r="T535" s="8"/>
       <c r="U535" s="8"/>
       <c r="V535" s="42" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="536" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -24277,7 +24277,7 @@
       <c r="T536" s="8"/>
       <c r="U536" s="8"/>
       <c r="V536" s="42" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="537" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -24380,7 +24380,7 @@
       <c r="T539" s="8"/>
       <c r="U539" s="8"/>
       <c r="V539" s="42" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="540" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -24701,7 +24701,7 @@
         <v>85</v>
       </c>
       <c r="T548" s="8" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="U548" s="8"/>
       <c r="V548" s="42"/>
@@ -24876,7 +24876,7 @@
         <v>85</v>
       </c>
       <c r="T553" s="8" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="U553" s="8"/>
       <c r="V553" s="42"/>
@@ -25218,7 +25218,7 @@
       <c r="T563" s="8"/>
       <c r="U563" s="8"/>
       <c r="V563" s="42" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="564" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -25321,7 +25321,7 @@
       <c r="T566" s="8"/>
       <c r="U566" s="8"/>
       <c r="V566" s="42" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="567" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -25655,7 +25655,7 @@
       <c r="T576" s="8"/>
       <c r="U576" s="8"/>
       <c r="V576" s="42" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="577" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -25955,7 +25955,7 @@
       <c r="T585" s="8"/>
       <c r="U585" s="8"/>
       <c r="V585" s="42" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="586" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -26466,7 +26466,7 @@
       <c r="T600" s="8"/>
       <c r="U600" s="8"/>
       <c r="V600" s="42" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="601" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -26536,7 +26536,7 @@
       <c r="T602" s="8"/>
       <c r="U602" s="8"/>
       <c r="V602" s="42" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="603" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -26738,7 +26738,7 @@
       <c r="T608" s="8"/>
       <c r="U608" s="8"/>
       <c r="V608" s="42" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="609" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -26911,7 +26911,7 @@
       <c r="T613" s="8"/>
       <c r="U613" s="8"/>
       <c r="V613" s="42" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="614" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -26981,7 +26981,7 @@
         <v>111</v>
       </c>
       <c r="T615" s="8" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="U615" s="8"/>
       <c r="V615" s="42"/>
@@ -27053,7 +27053,7 @@
       <c r="T617" s="8"/>
       <c r="U617" s="8"/>
       <c r="V617" s="42" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="618" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -27191,7 +27191,7 @@
       <c r="T621" s="8"/>
       <c r="U621" s="8"/>
       <c r="V621" s="42" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="622" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -27411,7 +27411,7 @@
       <c r="T627" s="8"/>
       <c r="U627" s="8"/>
       <c r="V627" s="42" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="628" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -27551,7 +27551,7 @@
       <c r="T631" s="18"/>
       <c r="U631" s="18"/>
       <c r="V631" s="42" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="632" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -27918,7 +27918,7 @@
       <c r="T642" s="8"/>
       <c r="U642" s="8"/>
       <c r="V642" s="42" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="643" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -28088,7 +28088,7 @@
       <c r="T647" s="8"/>
       <c r="U647" s="8"/>
       <c r="V647" s="42" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="648" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -28264,7 +28264,7 @@
       <c r="T652" s="8"/>
       <c r="U652" s="8"/>
       <c r="V652" s="42" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="653" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -28367,7 +28367,7 @@
       <c r="T655" s="8"/>
       <c r="U655" s="8"/>
       <c r="V655" s="42" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="656" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -28571,7 +28571,7 @@
       <c r="T661" s="8"/>
       <c r="U661" s="8"/>
       <c r="V661" s="42" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="662" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -28641,7 +28641,7 @@
       <c r="T663" s="8"/>
       <c r="U663" s="8"/>
       <c r="V663" s="42" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="664" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -28777,7 +28777,7 @@
       <c r="T667" s="8"/>
       <c r="U667" s="8"/>
       <c r="V667" s="42" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="668" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -28812,7 +28812,7 @@
       <c r="T668" s="8"/>
       <c r="U668" s="8"/>
       <c r="V668" s="42" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="669" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -28847,7 +28847,7 @@
       <c r="T669" s="8"/>
       <c r="U669" s="8"/>
       <c r="V669" s="42" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="670" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -28882,7 +28882,7 @@
       <c r="T670" s="8"/>
       <c r="U670" s="8"/>
       <c r="V670" s="42" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="671" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29010,7 +29010,7 @@
       <c r="T674" s="8"/>
       <c r="U674" s="8"/>
       <c r="V674" s="42" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="675" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29045,7 +29045,7 @@
       <c r="T675" s="8"/>
       <c r="U675" s="8"/>
       <c r="V675" s="42" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="676" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29111,7 +29111,7 @@
       <c r="T677" s="8"/>
       <c r="U677" s="8"/>
       <c r="V677" s="42" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="678" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29134,7 +29134,7 @@
         <v>36</v>
       </c>
       <c r="N678" s="43" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="O678" s="8" t="s">
         <v>64</v>
@@ -29146,7 +29146,7 @@
       <c r="T678" s="8"/>
       <c r="U678" s="8"/>
       <c r="V678" s="42" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="679" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29181,7 +29181,7 @@
       <c r="T679" s="8"/>
       <c r="U679" s="8"/>
       <c r="V679" s="42" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="680" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29216,7 +29216,7 @@
       <c r="T680" s="8"/>
       <c r="U680" s="8"/>
       <c r="V680" s="42" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="681" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29251,7 +29251,7 @@
       <c r="T681" s="8"/>
       <c r="U681" s="8"/>
       <c r="V681" s="42" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="682" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29348,7 +29348,7 @@
       <c r="T684" s="8"/>
       <c r="U684" s="8"/>
       <c r="V684" s="42" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="685" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29542,7 +29542,7 @@
       <c r="T690" s="8"/>
       <c r="U690" s="8"/>
       <c r="V690" s="42" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="691" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29766,7 +29766,7 @@
       <c r="T697" s="8"/>
       <c r="U697" s="8"/>
       <c r="V697" s="42" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="698" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29863,7 +29863,7 @@
       <c r="T700" s="8"/>
       <c r="U700" s="8"/>
       <c r="V700" s="42" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="701" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -29929,7 +29929,7 @@
       <c r="T702" s="8"/>
       <c r="U702" s="8"/>
       <c r="V702" s="42" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="703" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -30026,7 +30026,7 @@
       <c r="T705" s="8"/>
       <c r="U705" s="8"/>
       <c r="V705" s="42" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="706" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -30061,7 +30061,7 @@
       <c r="T706" s="8"/>
       <c r="U706" s="8"/>
       <c r="V706" s="42" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="707" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -30158,7 +30158,7 @@
       <c r="T709" s="8"/>
       <c r="U709" s="8"/>
       <c r="V709" s="42" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="710" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -30255,7 +30255,7 @@
       <c r="T712" s="8"/>
       <c r="U712" s="8"/>
       <c r="V712" s="42" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="713" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -30352,7 +30352,7 @@
       <c r="T715" s="8"/>
       <c r="U715" s="8"/>
       <c r="V715" s="42" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="716" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -30543,7 +30543,7 @@
       <c r="T721" s="8"/>
       <c r="U721" s="8"/>
       <c r="V721" s="42" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="722" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -30766,7 +30766,7 @@
       <c r="T728" s="8"/>
       <c r="U728" s="8"/>
       <c r="V728" s="42" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="729" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -30866,7 +30866,7 @@
       <c r="T731" s="8"/>
       <c r="U731" s="8"/>
       <c r="V731" s="42" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="732" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -30966,7 +30966,7 @@
       <c r="T734" s="8"/>
       <c r="U734" s="8"/>
       <c r="V734" s="42" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="735" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -31210,7 +31210,7 @@
         <v>100</v>
       </c>
       <c r="N742" s="43" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="O742" s="8" t="s">
         <v>64</v>
@@ -31222,7 +31222,7 @@
       <c r="T742" s="8"/>
       <c r="U742" s="8"/>
       <c r="V742" s="43" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="743" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -31349,7 +31349,7 @@
       <c r="T746" s="8"/>
       <c r="U746" s="8"/>
       <c r="V746" s="42" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="747" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -31384,7 +31384,7 @@
       <c r="T747" s="8"/>
       <c r="U747" s="8"/>
       <c r="V747" s="42" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="748" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -31419,7 +31419,7 @@
       <c r="T748" s="8"/>
       <c r="U748" s="8"/>
       <c r="V748" s="42" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="749" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -31516,7 +31516,7 @@
       <c r="T751" s="8"/>
       <c r="U751" s="8"/>
       <c r="V751" s="42" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="752" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -31551,7 +31551,7 @@
       <c r="T752" s="8"/>
       <c r="U752" s="8"/>
       <c r="V752" s="42" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="753" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -31805,7 +31805,7 @@
       <c r="T760" s="8"/>
       <c r="U760" s="8"/>
       <c r="V760" s="42" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="761" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -31968,7 +31968,7 @@
       <c r="T765" s="8"/>
       <c r="U765" s="8"/>
       <c r="V765" s="42" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="766" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -32222,7 +32222,7 @@
       <c r="T773" s="8"/>
       <c r="U773" s="8"/>
       <c r="V773" s="42" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="774" spans="6:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -32291,7 +32291,7 @@
       <c r="T775" s="8"/>
       <c r="U775" s="8"/>
       <c r="V775" s="42" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="776" spans="6:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -32642,7 +32642,7 @@
       <c r="T786" s="8"/>
       <c r="U786" s="8"/>
       <c r="V786" s="42" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="787" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -33170,7 +33170,7 @@
       <c r="T802" s="8"/>
       <c r="U802" s="8"/>
       <c r="V802" s="42" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="803" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -33346,7 +33346,7 @@
       <c r="T807" s="8"/>
       <c r="U807" s="8"/>
       <c r="V807" s="42" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="808" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -33384,7 +33384,7 @@
       <c r="T808" s="8"/>
       <c r="U808" s="8"/>
       <c r="V808" s="42" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="809" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -33496,7 +33496,7 @@
       <c r="T811" s="8"/>
       <c r="U811" s="8"/>
       <c r="V811" s="42" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="812" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -33540,7 +33540,7 @@
       <c r="T812" s="8"/>
       <c r="U812" s="8"/>
       <c r="V812" s="42" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="813" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -33584,7 +33584,7 @@
       <c r="T813" s="8"/>
       <c r="U813" s="8"/>
       <c r="V813" s="42" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="814" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -33746,7 +33746,7 @@
       <c r="T818" s="8"/>
       <c r="U818" s="8"/>
       <c r="V818" s="42" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="819" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -33818,7 +33818,7 @@
       <c r="T820" s="8"/>
       <c r="U820" s="8"/>
       <c r="V820" s="42" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="821" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -34079,7 +34079,7 @@
       <c r="T828" s="8"/>
       <c r="U828" s="8"/>
       <c r="V828" s="42" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="829" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -34364,7 +34364,7 @@
         <v>111</v>
       </c>
       <c r="T837" s="8" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="U837" s="8"/>
       <c r="V837" s="42"/>
@@ -35201,7 +35201,7 @@
       <c r="T863" s="8"/>
       <c r="U863" s="8"/>
       <c r="V863" s="42" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="864" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -35236,7 +35236,7 @@
       <c r="T864" s="8"/>
       <c r="U864" s="8"/>
       <c r="V864" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="865" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -35333,7 +35333,7 @@
       <c r="T867" s="8"/>
       <c r="U867" s="8"/>
       <c r="V867" s="42" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="868" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -35389,7 +35389,7 @@
         <v>227</v>
       </c>
       <c r="N869" s="43" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="O869" s="7"/>
       <c r="P869" s="8"/>
@@ -35656,7 +35656,7 @@
       <c r="T877" s="8"/>
       <c r="U877" s="8"/>
       <c r="V877" s="42" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="878" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -35882,7 +35882,7 @@
       <c r="T884" s="8"/>
       <c r="U884" s="8"/>
       <c r="V884" s="42" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="885" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -35917,7 +35917,7 @@
       <c r="T885" s="8"/>
       <c r="U885" s="8"/>
       <c r="V885" s="42" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="886" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -35983,7 +35983,7 @@
       <c r="T887" s="8"/>
       <c r="U887" s="8"/>
       <c r="V887" s="42" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="888" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -36018,7 +36018,7 @@
       <c r="T888" s="8"/>
       <c r="U888" s="8"/>
       <c r="V888" s="42" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="889" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -36084,7 +36084,7 @@
       <c r="T890" s="8"/>
       <c r="U890" s="8"/>
       <c r="V890" s="42" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="891" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -36890,7 +36890,7 @@
       <c r="T915" s="8"/>
       <c r="U915" s="8"/>
       <c r="V915" s="42" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="916" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -36956,7 +36956,7 @@
       <c r="T917" s="8"/>
       <c r="U917" s="8"/>
       <c r="V917" s="42" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="918" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -37086,7 +37086,7 @@
       <c r="T921" s="8"/>
       <c r="U921" s="8"/>
       <c r="V921" s="42" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="922" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -37109,7 +37109,7 @@
         <v>280</v>
       </c>
       <c r="N922" s="42" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="O922" s="8" t="s">
         <v>64</v>
@@ -37123,7 +37123,7 @@
       <c r="T922" s="8"/>
       <c r="U922" s="8"/>
       <c r="V922" s="42" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="923" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -37156,7 +37156,7 @@
       <c r="T923" s="8"/>
       <c r="U923" s="8"/>
       <c r="V923" s="42" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="924" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -37191,7 +37191,7 @@
       <c r="T924" s="8"/>
       <c r="U924" s="8"/>
       <c r="V924" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="925" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -37722,7 +37722,7 @@
       <c r="T941" s="8"/>
       <c r="U941" s="8"/>
       <c r="V941" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="942" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -39181,7 +39181,7 @@
       <c r="T987" s="8"/>
       <c r="U987" s="8"/>
       <c r="V987" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="988" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -39280,7 +39280,7 @@
       <c r="T990" s="8"/>
       <c r="U990" s="8"/>
       <c r="V990" s="42" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="991" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -39346,7 +39346,7 @@
       <c r="T992" s="8"/>
       <c r="U992" s="8"/>
       <c r="V992" s="42" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="993" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -39416,7 +39416,7 @@
       <c r="T994" s="8"/>
       <c r="U994" s="8"/>
       <c r="V994" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="995" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -39451,7 +39451,7 @@
       <c r="T995" s="8"/>
       <c r="U995" s="8"/>
       <c r="V995" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="996" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -39915,7 +39915,7 @@
       <c r="T1009" s="8"/>
       <c r="U1009" s="8"/>
       <c r="V1009" s="42" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="1010" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -39951,7 +39951,7 @@
       <c r="T1010" s="8"/>
       <c r="U1010" s="8"/>
       <c r="V1010" s="42" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="1011" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -40025,7 +40025,7 @@
       <c r="T1012" s="8"/>
       <c r="U1012" s="8"/>
       <c r="V1012" s="42" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="1013" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -40444,7 +40444,7 @@
       <c r="T1025" s="8"/>
       <c r="U1025" s="8"/>
       <c r="V1025" s="42" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="1026" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -40543,7 +40543,7 @@
       <c r="T1028" s="8"/>
       <c r="U1028" s="8"/>
       <c r="V1028" s="42" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="1029" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -40926,7 +40926,7 @@
       <c r="T1040" s="8"/>
       <c r="U1040" s="8"/>
       <c r="V1040" s="42" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="1041" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -41042,7 +41042,7 @@
     </row>
     <row r="1044" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A1044" s="8" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="E1044" s="50" t="s">
         <v>114</v>
@@ -41433,7 +41433,7 @@
       <c r="T1055" s="8"/>
       <c r="U1055" s="8"/>
       <c r="V1055" s="42" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="1056" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -41594,7 +41594,7 @@
       <c r="T1060" s="8"/>
       <c r="U1060" s="8"/>
       <c r="V1060" s="42" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="1061" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -42066,7 +42066,7 @@
       <c r="T1075" s="8"/>
       <c r="U1075" s="8"/>
       <c r="V1075" s="42" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="1076" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -42228,7 +42228,7 @@
       <c r="T1080" s="8"/>
       <c r="U1080" s="8"/>
       <c r="V1080" s="42" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="1081" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -42425,7 +42425,7 @@
       <c r="T1086" s="8"/>
       <c r="U1086" s="8"/>
       <c r="V1086" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="1087" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -42557,7 +42557,7 @@
       <c r="T1090" s="8"/>
       <c r="U1090" s="8"/>
       <c r="V1090" s="42" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="1091" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -42593,7 +42593,7 @@
       <c r="T1091" s="8"/>
       <c r="U1091" s="8"/>
       <c r="V1091" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="1092" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -42722,7 +42722,7 @@
       <c r="T1095" s="8"/>
       <c r="U1095" s="8"/>
       <c r="V1095" s="42" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="1096" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -42821,7 +42821,7 @@
       <c r="T1098" s="8"/>
       <c r="U1098" s="8"/>
       <c r="V1098" s="42" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="1099" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -42857,7 +42857,7 @@
       <c r="T1099" s="8"/>
       <c r="U1099" s="8"/>
       <c r="V1099" s="42" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="1100" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -43087,7 +43087,7 @@
       <c r="T1106" s="8"/>
       <c r="U1106" s="8"/>
       <c r="V1106" s="42" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="1107" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -43154,7 +43154,7 @@
       <c r="T1108" s="8"/>
       <c r="U1108" s="8"/>
       <c r="V1108" s="42" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="1109" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -43177,7 +43177,7 @@
         <v>187</v>
       </c>
       <c r="N1109" s="42" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="O1109" s="8" t="s">
         <v>64</v>
@@ -43191,7 +43191,7 @@
       <c r="T1109" s="8"/>
       <c r="U1109" s="8"/>
       <c r="V1109" s="42" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="1110" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -43379,7 +43379,7 @@
       <c r="T1115" s="8"/>
       <c r="U1115" s="8"/>
       <c r="V1115" s="42" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="1116" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -43593,7 +43593,7 @@
         <v>13</v>
       </c>
       <c r="N1122" s="43" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="O1122" s="8" t="s">
         <v>64</v>
@@ -43605,7 +43605,7 @@
       <c r="T1122" s="8"/>
       <c r="U1122" s="8"/>
       <c r="V1122" s="42" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="1123" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -43640,7 +43640,7 @@
       <c r="T1123" s="8"/>
       <c r="U1123" s="8"/>
       <c r="V1123" s="42" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="1124" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -43675,7 +43675,7 @@
       <c r="T1124" s="8"/>
       <c r="U1124" s="8"/>
       <c r="V1124" s="42" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="1125" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -44055,7 +44055,7 @@
       <c r="T1136" s="8"/>
       <c r="U1136" s="8"/>
       <c r="V1136" s="42" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="1137" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -44217,12 +44217,12 @@
       <c r="T1141" s="8"/>
       <c r="U1141" s="8"/>
       <c r="V1141" s="42" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="1142" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A1142" s="8" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="I1142" s="45" t="s">
         <v>43</v>
@@ -44446,7 +44446,7 @@
       <c r="T1148" s="8"/>
       <c r="U1148" s="8"/>
       <c r="V1148" s="42" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="1149" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -44482,7 +44482,7 @@
       <c r="T1149" s="8"/>
       <c r="U1149" s="8"/>
       <c r="V1149" s="42" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="1150" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -44619,7 +44619,7 @@
       <c r="T1153" s="8"/>
       <c r="U1153" s="8"/>
       <c r="V1153" s="42" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="1154" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -44973,7 +44973,7 @@
       <c r="T1164" s="8"/>
       <c r="U1164" s="8"/>
       <c r="V1164" s="42" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="1165" spans="4:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -45954,7 +45954,7 @@
       <c r="T1195" s="8"/>
       <c r="U1195" s="8"/>
       <c r="V1195" s="42" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="1196" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -46142,7 +46142,7 @@
       <c r="T1201" s="8"/>
       <c r="U1201" s="8"/>
       <c r="V1201" s="42" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="1202" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -46305,7 +46305,7 @@
     </row>
     <row r="1207" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A1207" s="62" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="B1207" s="63"/>
       <c r="C1207" s="51"/>
@@ -46345,7 +46345,7 @@
       <c r="T1207" s="8"/>
       <c r="U1207" s="8"/>
       <c r="V1207" s="42" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="1208" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -46538,7 +46538,7 @@
       <c r="T1213" s="8"/>
       <c r="U1213" s="8"/>
       <c r="V1213" s="42" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="1214" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -46716,7 +46716,7 @@
         <v>24</v>
       </c>
       <c r="N1219" s="43" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="O1219" s="8" t="s">
         <v>64</v>
@@ -46728,7 +46728,7 @@
       <c r="T1219" s="8"/>
       <c r="U1219" s="8"/>
       <c r="V1219" s="42" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="1220" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -46794,7 +46794,7 @@
       <c r="T1221" s="8"/>
       <c r="U1221" s="8"/>
       <c r="V1221" s="42" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="1222" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -47112,7 +47112,7 @@
       <c r="T1231" s="8"/>
       <c r="U1231" s="8"/>
       <c r="V1231" s="42" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="1232" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -47136,7 +47136,7 @@
         <v>37</v>
       </c>
       <c r="N1232" s="43" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="O1232" s="8" t="s">
         <v>64</v>
@@ -47148,7 +47148,7 @@
       <c r="T1232" s="8"/>
       <c r="U1232" s="8"/>
       <c r="V1232" s="42" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="1233" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -47214,7 +47214,7 @@
       <c r="T1234" s="8"/>
       <c r="U1234" s="8"/>
       <c r="V1234" s="42" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="1235" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -47404,7 +47404,7 @@
       <c r="T1240" s="8"/>
       <c r="U1240" s="8"/>
       <c r="V1240" s="42" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="1241" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -47905,7 +47905,7 @@
       <c r="T1256" s="8"/>
       <c r="U1256" s="8"/>
       <c r="V1256" s="42" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="1257" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -47940,7 +47940,7 @@
       <c r="T1257" s="8"/>
       <c r="U1257" s="8"/>
       <c r="V1257" s="42" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="1258" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -48006,7 +48006,7 @@
       <c r="T1259" s="8"/>
       <c r="U1259" s="8"/>
       <c r="V1259" s="42" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="1260" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -48233,7 +48233,7 @@
       <c r="T1266" s="8"/>
       <c r="U1266" s="8"/>
       <c r="V1266" s="42" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="1267" spans="5:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -48432,7 +48432,7 @@
       <c r="T1272" s="8"/>
       <c r="U1272" s="8"/>
       <c r="V1272" s="42" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="1273" spans="5:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -48686,7 +48686,7 @@
       <c r="T1280" s="8"/>
       <c r="U1280" s="8"/>
       <c r="V1280" s="42" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="1281" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -48802,7 +48802,7 @@
         <v>89</v>
       </c>
       <c r="N1284" s="42" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="O1284" s="8" t="s">
         <v>64</v>
@@ -48815,10 +48815,10 @@
       <c r="S1284" s="8"/>
       <c r="T1284" s="8"/>
       <c r="U1284" s="8" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="V1284" s="42" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="1285" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -49224,7 +49224,7 @@
       <c r="T1297" s="8"/>
       <c r="U1297" s="8"/>
       <c r="V1297" s="42" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="1298" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -49354,7 +49354,7 @@
       <c r="T1301" s="8"/>
       <c r="U1301" s="8"/>
       <c r="V1301" s="42" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="1302" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -49558,7 +49558,7 @@
       <c r="T1307" s="8"/>
       <c r="U1307" s="8"/>
       <c r="V1307" s="42" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="1308" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -50038,7 +50038,7 @@
         <v>127</v>
       </c>
       <c r="N1322" s="43" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="O1322" s="8" t="s">
         <v>64</v>
@@ -50050,7 +50050,7 @@
       <c r="T1322" s="8"/>
       <c r="U1322" s="8"/>
       <c r="V1322" s="42" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="1323" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -50118,7 +50118,7 @@
       <c r="T1324" s="8"/>
       <c r="U1324" s="8"/>
       <c r="V1324" s="42" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="1325" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -50155,7 +50155,7 @@
       <c r="T1325" s="8"/>
       <c r="U1325" s="8"/>
       <c r="V1325" s="42" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="1326" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -50291,7 +50291,7 @@
       <c r="T1329" s="8"/>
       <c r="U1329" s="8"/>
       <c r="V1329" s="42" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="1330" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -50395,7 +50395,7 @@
       <c r="S1332" s="8"/>
       <c r="T1332" s="8"/>
       <c r="V1332" s="42" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="1333" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -50425,7 +50425,7 @@
         <v>138</v>
       </c>
       <c r="N1333" s="53" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="O1333" s="7"/>
       <c r="P1333" s="8"/>
@@ -50534,7 +50534,7 @@
         <v>141</v>
       </c>
       <c r="N1336" s="53" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="O1336" s="8"/>
       <c r="P1336" s="8"/>
@@ -50712,7 +50712,7 @@
       <c r="T1341" s="8"/>
       <c r="U1341" s="8"/>
       <c r="V1341" s="42" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="1342" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -50780,7 +50780,7 @@
       <c r="T1343" s="8"/>
       <c r="U1343" s="8"/>
       <c r="V1343" s="42" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="1344" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -50911,7 +50911,7 @@
       <c r="T1347" s="8"/>
       <c r="U1347" s="8"/>
       <c r="V1347" s="42" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="1348" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -51011,7 +51011,7 @@
       <c r="T1350" s="8"/>
       <c r="U1350" s="8"/>
       <c r="V1350" s="42" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="1351" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -51340,7 +51340,7 @@
       <c r="T1360" s="8"/>
       <c r="U1360" s="8"/>
       <c r="V1360" s="42" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="1361" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -51410,7 +51410,7 @@
       <c r="T1362" s="8"/>
       <c r="U1362" s="8"/>
       <c r="V1362" s="42" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="1363" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -51576,7 +51576,7 @@
       <c r="T1367" s="8"/>
       <c r="U1367" s="8"/>
       <c r="V1367" s="42" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="1368" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -51647,7 +51647,7 @@
       <c r="T1369" s="8"/>
       <c r="U1369" s="8"/>
       <c r="V1369" s="43" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="1370" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -51750,7 +51750,7 @@
       <c r="T1372" s="8"/>
       <c r="U1372" s="8"/>
       <c r="V1372" s="42" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="1373" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -51819,7 +51819,7 @@
       <c r="T1374" s="8"/>
       <c r="U1374" s="8"/>
       <c r="V1374" s="42" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="1375" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -51887,7 +51887,7 @@
       <c r="T1376" s="8"/>
       <c r="U1376" s="8"/>
       <c r="V1376" s="42" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="1377" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -52280,7 +52280,7 @@
       <c r="T1388" s="8"/>
       <c r="U1388" s="8"/>
       <c r="V1388" s="42" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="1389" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -52348,7 +52348,7 @@
       <c r="T1390" s="8"/>
       <c r="U1390" s="8"/>
       <c r="V1390" s="42" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="1391" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -52446,7 +52446,7 @@
         <v>85</v>
       </c>
       <c r="T1393" s="8" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="U1393" s="8"/>
       <c r="V1393" s="42"/>
@@ -52550,7 +52550,7 @@
       <c r="T1396" s="8"/>
       <c r="U1396" s="8"/>
       <c r="V1396" s="42" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="1397" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -52622,7 +52622,7 @@
       <c r="T1398" s="8"/>
       <c r="U1398" s="8"/>
       <c r="V1398" s="42" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="1399" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -52722,7 +52722,7 @@
       <c r="T1401" s="8"/>
       <c r="U1401" s="8"/>
       <c r="V1401" s="42" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="1402" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -52824,7 +52824,7 @@
     </row>
     <row r="1405" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A1405" s="8" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="C1405" s="37"/>
       <c r="F1405" s="50" t="s">
@@ -53035,7 +53035,7 @@
       <c r="T1410" s="8"/>
       <c r="U1410" s="8"/>
       <c r="V1410" s="42" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="1411" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -53103,7 +53103,7 @@
       <c r="T1412" s="8"/>
       <c r="U1412" s="8"/>
       <c r="V1412" s="42" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="1413" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -53203,7 +53203,7 @@
       <c r="T1415" s="8"/>
       <c r="U1415" s="8"/>
       <c r="V1415" s="42" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="1416" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -53239,7 +53239,7 @@
       <c r="T1416" s="8"/>
       <c r="U1416" s="8"/>
       <c r="V1416" s="42" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="1417" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -53307,7 +53307,7 @@
       <c r="T1418" s="8"/>
       <c r="U1418" s="8"/>
       <c r="V1418" s="42" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="1419" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -53727,7 +53727,7 @@
       <c r="T1431" s="8"/>
       <c r="U1431" s="8"/>
       <c r="V1431" s="42" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="1432" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -53795,7 +53795,7 @@
       <c r="T1433" s="8"/>
       <c r="U1433" s="8"/>
       <c r="V1433" s="42" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="1434" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -53959,7 +53959,7 @@
       <c r="T1438" s="8"/>
       <c r="U1438" s="8"/>
       <c r="V1438" s="42" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="1439" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -53995,7 +53995,7 @@
       <c r="T1439" s="8"/>
       <c r="U1439" s="8"/>
       <c r="V1439" s="42" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="1440" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -54512,7 +54512,7 @@
       <c r="T1455" s="8"/>
       <c r="U1455" s="8"/>
       <c r="V1455" s="42" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="1456" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -54616,7 +54616,7 @@
       <c r="T1458" s="8"/>
       <c r="U1458" s="8"/>
       <c r="V1458" s="42" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="1459" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -54654,7 +54654,7 @@
       <c r="T1459" s="8"/>
       <c r="U1459" s="8"/>
       <c r="V1459" s="42" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="1460" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -54760,7 +54760,7 @@
       <c r="T1462" s="8"/>
       <c r="U1462" s="8"/>
       <c r="V1462" s="42" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="1463" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -54796,7 +54796,7 @@
       <c r="T1463" s="8"/>
       <c r="U1463" s="8"/>
       <c r="V1463" s="42" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="1464" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -54896,7 +54896,7 @@
       <c r="T1466" s="8"/>
       <c r="U1466" s="8"/>
       <c r="V1466" s="42" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="1467" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -55161,7 +55161,7 @@
       <c r="T1474" s="8"/>
       <c r="U1474" s="8"/>
       <c r="V1474" s="42" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="1475" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -55231,7 +55231,7 @@
       <c r="T1476" s="8"/>
       <c r="U1476" s="8"/>
       <c r="V1476" s="42" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="1477" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -55431,7 +55431,7 @@
       <c r="T1482" s="8"/>
       <c r="U1482" s="8"/>
       <c r="V1482" s="42" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="1483" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -55609,7 +55609,7 @@
       <c r="T1487" s="8"/>
       <c r="U1487" s="8"/>
       <c r="V1487" s="42" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="1488" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -55709,7 +55709,7 @@
       <c r="T1490" s="8"/>
       <c r="U1490" s="8"/>
       <c r="V1490" s="42" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="1491" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -55968,7 +55968,7 @@
       <c r="T1498" s="8"/>
       <c r="U1498" s="8"/>
       <c r="V1498" s="42" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="1499" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -56653,7 +56653,7 @@
       <c r="T1519" s="8"/>
       <c r="U1519" s="8"/>
       <c r="V1519" s="42" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="1520" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -56913,7 +56913,7 @@
       <c r="T1527" s="8"/>
       <c r="U1527" s="8"/>
       <c r="V1527" s="42" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="1528" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -57168,7 +57168,7 @@
       <c r="T1535" s="8"/>
       <c r="U1535" s="8"/>
       <c r="V1535" s="42" t="s">
-        <v>1221</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="1536" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -57513,7 +57513,7 @@
       <c r="T1546" s="8"/>
       <c r="U1546" s="8"/>
       <c r="V1546" s="42" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="1547" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -57579,7 +57579,7 @@
       <c r="T1548" s="8"/>
       <c r="U1548" s="8"/>
       <c r="V1548" s="42" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="1549" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -57923,7 +57923,7 @@
       <c r="T1559" s="8"/>
       <c r="U1559" s="8"/>
       <c r="V1559" s="42" t="s">
-        <v>1224</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="1560" spans="5:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -58113,7 +58113,7 @@
       <c r="T1565" s="8"/>
       <c r="U1565" s="8"/>
       <c r="V1565" s="42" t="s">
-        <v>1225</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="1566" spans="5:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -58816,13 +58816,13 @@
         <v>189</v>
       </c>
       <c r="N1590" s="42" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="P1590" s="8" t="s">
         <v>63</v>
       </c>
       <c r="V1590" s="42" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="1591" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -59803,7 +59803,7 @@
         <v>64</v>
       </c>
       <c r="V1630" s="42" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="1631" spans="7:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -60119,7 +60119,7 @@
         <v>64</v>
       </c>
       <c r="V1643" s="42" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="1644" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -60148,7 +60148,7 @@
         <v>64</v>
       </c>
       <c r="V1644" s="42" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="1645" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -60273,7 +60273,7 @@
         <v>64</v>
       </c>
       <c r="V1649" s="42" t="s">
-        <v>1229</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="1650" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -60326,7 +60326,7 @@
         <v>64</v>
       </c>
       <c r="V1651" s="42" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="1652" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -60646,7 +60646,7 @@
         <v>64</v>
       </c>
       <c r="V1664" s="42" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="1665" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -60819,7 +60819,7 @@
         <v>64</v>
       </c>
       <c r="V1671" s="42" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="1672" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -61157,7 +61157,7 @@
         <v>64</v>
       </c>
       <c r="V1684" s="42" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="1685" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -61294,7 +61294,7 @@
         <v>64</v>
       </c>
       <c r="V1689" s="42" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="1690" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -61670,7 +61670,7 @@
         <v>64</v>
       </c>
       <c r="V1704" s="42" t="s">
-        <v>1233</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="1705" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -61792,7 +61792,7 @@
         <v>119</v>
       </c>
       <c r="N1709" s="42" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
       <c r="O1709" s="8" t="s">
         <v>64</v>
@@ -61801,7 +61801,7 @@
         <v>63</v>
       </c>
       <c r="V1709" s="42" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="1710" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -61876,7 +61876,7 @@
         <v>64</v>
       </c>
       <c r="V1712" s="42" t="s">
-        <v>1234</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="1713" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -62001,7 +62001,7 @@
         <v>64</v>
       </c>
       <c r="V1717" s="42" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="1718" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -62390,7 +62390,7 @@
         <v>64</v>
       </c>
       <c r="V1733" s="42" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="1734" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -62704,7 +62704,7 @@
         <v>64</v>
       </c>
       <c r="V1745" s="42" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="1746" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -62733,7 +62733,7 @@
         <v>64</v>
       </c>
       <c r="V1746" s="42" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="1747" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -63005,7 +63005,7 @@
         <v>64</v>
       </c>
       <c r="V1757" s="42" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="1758" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -63228,7 +63228,7 @@
         <v>64</v>
       </c>
       <c r="V1766" s="42" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="1767" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -63281,7 +63281,7 @@
         <v>64</v>
       </c>
       <c r="V1768" s="42" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="1769" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -63334,7 +63334,7 @@
         <v>64</v>
       </c>
       <c r="V1770" s="42" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="1771" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -63483,7 +63483,7 @@
         <v>64</v>
       </c>
       <c r="V1776" s="42" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="1777" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -63584,7 +63584,7 @@
         <v>64</v>
       </c>
       <c r="V1780" s="42" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="1781" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64069,7 +64069,7 @@
         <v>64</v>
       </c>
       <c r="V1800" s="42" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="1801" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64452,7 +64452,7 @@
         <v>64</v>
       </c>
       <c r="V1814" s="42" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="1815" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64622,7 +64622,7 @@
         <v>64</v>
       </c>
       <c r="V1820" s="42" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="1821" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64675,7 +64675,7 @@
         <v>64</v>
       </c>
       <c r="V1822" s="42" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="1823" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64728,7 +64728,7 @@
         <v>64</v>
       </c>
       <c r="V1824" s="42" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="1825" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64856,7 +64856,7 @@
         <v>63</v>
       </c>
       <c r="V1829" s="42" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="1830" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64883,7 +64883,7 @@
         <v>64</v>
       </c>
       <c r="V1830" s="42" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="1831" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64960,7 +64960,7 @@
         <v>64</v>
       </c>
       <c r="V1833" s="42" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="1834" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -65109,7 +65109,7 @@
         <v>64</v>
       </c>
       <c r="V1839" s="42" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="1840" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -65765,7 +65765,7 @@
         <v>64</v>
       </c>
       <c r="V1865" s="42" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="1866" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -66082,7 +66082,7 @@
         <v>64</v>
       </c>
       <c r="V1878" s="42" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="1879" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -66449,7 +66449,7 @@
         <v>64</v>
       </c>
       <c r="V1892" s="42" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="1893" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -66678,7 +66678,7 @@
         <v>64</v>
       </c>
       <c r="V1901" s="42" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="1902" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -66779,7 +66779,7 @@
         <v>64</v>
       </c>
       <c r="V1905" s="42" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="1906" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -66850,13 +66850,13 @@
         <v>79</v>
       </c>
       <c r="N1908" s="43" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="O1908" s="8" t="s">
         <v>64</v>
       </c>
       <c r="V1908" s="43" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="1909" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -67520,7 +67520,7 @@
         <v>64</v>
       </c>
       <c r="V1935" s="42" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="1936" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -67669,7 +67669,7 @@
         <v>64</v>
       </c>
       <c r="V1941" s="42" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="1942" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -67797,7 +67797,7 @@
         <v>111</v>
       </c>
       <c r="T1946" s="8" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="V1946" s="42"/>
     </row>
@@ -67851,7 +67851,7 @@
         <v>64</v>
       </c>
       <c r="V1948" s="42" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="1949" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -67931,7 +67931,7 @@
         <v>64</v>
       </c>
       <c r="V1951" s="42" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="1952" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68059,7 +68059,7 @@
         <v>64</v>
       </c>
       <c r="V1956" s="42" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="1957" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68088,7 +68088,7 @@
         <v>64</v>
       </c>
       <c r="V1957" s="42" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="1958" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68237,7 +68237,7 @@
         <v>64</v>
       </c>
       <c r="V1963" s="42" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="1964" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68338,7 +68338,7 @@
         <v>64</v>
       </c>
       <c r="V1967" s="42" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="1968" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68514,7 +68514,7 @@
         <v>64</v>
       </c>
       <c r="V1974" s="42" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="1975" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68686,7 +68686,7 @@
         <v>64</v>
       </c>
       <c r="V1981" s="42" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="1982" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68766,7 +68766,7 @@
         <v>111</v>
       </c>
       <c r="T1984" s="8" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="V1984" s="42"/>
     </row>
@@ -68820,7 +68820,7 @@
         <v>64</v>
       </c>
       <c r="V1986" s="42" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="1987" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68849,7 +68849,7 @@
         <v>64</v>
       </c>
       <c r="V1987" s="42" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="1988" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69070,7 +69070,7 @@
         <v>64</v>
       </c>
       <c r="V1996" s="42" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="1997" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69198,7 +69198,7 @@
         <v>64</v>
       </c>
       <c r="V2001" s="42" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="2002" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69275,7 +69275,7 @@
         <v>64</v>
       </c>
       <c r="V2004" s="42" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="2005" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69376,7 +69376,7 @@
         <v>64</v>
       </c>
       <c r="V2008" s="42" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="2009" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69624,7 +69624,7 @@
         <v>111</v>
       </c>
       <c r="T2018" s="8" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="V2018" s="42"/>
     </row>
@@ -69702,7 +69702,7 @@
         <v>64</v>
       </c>
       <c r="V2021" s="42" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="2022" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69808,7 +69808,7 @@
         <v>64</v>
       </c>
       <c r="V2025" s="42" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="2026" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -70280,7 +70280,7 @@
     </row>
     <row r="2045" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A2045" s="64" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="H2045" s="49" t="s">
         <v>108</v>
@@ -70705,7 +70705,7 @@
         <v>64</v>
       </c>
       <c r="V2060" s="42" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="2061" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71195,7 +71195,7 @@
         <v>64</v>
       </c>
       <c r="V2080" s="42" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="2081" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71323,7 +71323,7 @@
         <v>66</v>
       </c>
       <c r="V2085" s="42" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="2086" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71352,7 +71352,7 @@
         <v>67</v>
       </c>
       <c r="V2086" s="42" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="2087" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71381,7 +71381,7 @@
         <v>64</v>
       </c>
       <c r="V2087" s="42" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="2088" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71491,7 +71491,7 @@
         <v>64</v>
       </c>
       <c r="V2091" s="42" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="2092" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71658,7 +71658,7 @@
         <v>64</v>
       </c>
       <c r="V2097" s="42" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="2098" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71711,7 +71711,7 @@
         <v>64</v>
       </c>
       <c r="V2099" s="42" t="s">
-        <v>1270</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="2100" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71764,7 +71764,7 @@
         <v>64</v>
       </c>
       <c r="V2101" s="42" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="2102" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71793,7 +71793,7 @@
         <v>64</v>
       </c>
       <c r="V2102" s="42" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="2103" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71894,7 +71894,7 @@
         <v>64</v>
       </c>
       <c r="V2106" s="42" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="2107" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -72219,7 +72219,7 @@
         <v>64</v>
       </c>
       <c r="V2119" s="42" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="2120" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -72386,7 +72386,7 @@
         <v>297</v>
       </c>
       <c r="N2126" s="56" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="O2126" s="8" t="s">
         <v>64</v>
@@ -72395,7 +72395,7 @@
         <v>63</v>
       </c>
       <c r="V2126" s="43" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>